<commit_message>
test: expand USB and event review journey coverage
Require USB discovery, preview, inference and restart checks. Add event-report
review cases for local and OpenAI-compatible models, including target-specific
positive/negative checks, prompt changes and recoverable interface failures.
Retain device-log download coverage, add VLM memory-pressure recovery coverage,
and align MQTT expectations with the HTTP-alert/MQTT-control design.

Update the full and quick XLSX casebooks, generated suite mirrors, resource
example and documentation. Keep service endpoints and credentials private.

Validation: both suite compile checks and schema validation passed, all 32
journey-tool tests passed, and docs:verify passed. New case definitions remain
unexecuted and do not overwrite historical device results.
</commit_message>
<xml_diff>
--- a/test/customer-journey/CosmoEdge-主要功能客户旅程测试用例.xlsx
+++ b/test/customer-journey/CosmoEdge-主要功能客户旅程测试用例.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评审总览" sheetId="1" r:id="R50abca8c7092439a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主要用例" sheetId="2" r:id="R56cf9666b22348bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤与验收" sheetId="3" r:id="R0820840be99b4cc2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="按需补测" sheetId="4" r:id="Ra60342abbb694fb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="范围与评审" sheetId="5" r:id="Rce831478a36b44a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评审总览" sheetId="1" r:id="R4e2e12dec86c44b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主要用例" sheetId="2" r:id="Reb05f24b4b734d80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤与验收" sheetId="3" r:id="R23f294e649194cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="按需补测" sheetId="4" r:id="Ra763ecfcb5974a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="范围与评审" sheetId="5" r:id="R9023807993d24ff5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -146,7 +146,7 @@
         <x:color rgb="FF9A3412"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4E4"/>
         </x:patternFill>
       </x:fill>
@@ -157,7 +157,7 @@
         <x:color rgb="FF9A3412"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D5"/>
         </x:patternFill>
       </x:fill>
@@ -168,7 +168,7 @@
         <x:color rgb="FF9A3412"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0D5"/>
         </x:patternFill>
       </x:fill>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QuickCases" displayName="QuickCases" ref="A4:L32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QuickCases" displayName="QuickCases" ref="A4:L33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L33"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="模块"/>
@@ -199,8 +199,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuickSteps" displayName="QuickSteps" ref="A4:I99" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:I99"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="QuickSteps" displayName="QuickSteps" ref="A4:I106" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:I106"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="用例编号"/>
     <x:tableColumn id="2" name="步骤编号"/>
@@ -472,7 +472,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="str">
-        <x:v>v0.5 已确认快测用例 · 2026-10-14 · 尚未执行设备测试</x:v>
+        <x:v>v0.7 已确认快测用例 · 2026-10-19 · 用例定义，实测结果另存</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -493,15 +493,15 @@
         <x:v>核心用例数</x:v>
       </x:c>
       <x:c r="B5" s="3" t="n">
-        <x:f>COUNTA('主要用例'!A5:A32)</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTA('主要用例'!A5:A33)</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
       <x:c r="D5" s="3" t="str">
         <x:v>通过</x:v>
       </x:c>
       <x:c r="E5" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"通过")</x:f>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"通过")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F5" s="15" t="str">
@@ -513,14 +513,14 @@
         <x:v>逐步验收数</x:v>
       </x:c>
       <x:c r="B6" s="3" t="n">
-        <x:v>95</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="3" t="str">
         <x:v>失败</x:v>
       </x:c>
       <x:c r="E6" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"失败")</x:f>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"失败")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="15" t="str">
@@ -532,15 +532,15 @@
         <x:v>预计正常下限（分钟）</x:v>
       </x:c>
       <x:c r="B7" s="3" t="n">
-        <x:f>SUM('主要用例'!F5:F32)</x:f>
-        <x:v>141</x:v>
+        <x:f>SUM('主要用例'!F5:F33)</x:f>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3" t="str">
         <x:v>阻塞</x:v>
       </x:c>
       <x:c r="E7" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"阻塞")</x:f>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"阻塞")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="3" t="str">
@@ -552,15 +552,15 @@
         <x:v>预计正常上限（分钟）</x:v>
       </x:c>
       <x:c r="B8" s="3" t="n">
-        <x:f>SUM('主要用例'!G5:G32)</x:f>
-        <x:v>232</x:v>
+        <x:f>SUM('主要用例'!G5:G33)</x:f>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3" t="str">
         <x:v>部分完成</x:v>
       </x:c>
       <x:c r="E8" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"部分完成")</x:f>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"部分完成")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="3" t="str">
@@ -579,8 +579,8 @@
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="E9" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"未执行")</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"未执行")</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F9" s="3"/>
     </x:row>
@@ -592,7 +592,7 @@
         <x:v>不适用</x:v>
       </x:c>
       <x:c r="E10" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!J5:J32,"不适用")</x:f>
+        <x:f>COUNTIFS('主要用例'!J5:J33,"不适用")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="3"/>
@@ -620,15 +620,15 @@
         <x:v>准备与登录</x:v>
       </x:c>
       <x:c r="B12" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A12)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A12)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C12" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A12)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A12)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D12" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A12)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A12)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E12" s="3"/>
@@ -641,15 +641,15 @@
         <x:v>模型与场景</x:v>
       </x:c>
       <x:c r="B13" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A13)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A13)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C13" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A13)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A13)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="D13" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A13)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A13)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="E13" s="3"/>
@@ -662,15 +662,15 @@
         <x:v>视频接入</x:v>
       </x:c>
       <x:c r="B14" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A14)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A14)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C14" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A14)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A14)</x:f>
         <x:v>29</x:v>
       </x:c>
       <x:c r="D14" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A14)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A14)</x:f>
         <x:v>46</x:v>
       </x:c>
       <x:c r="E14" s="3"/>
@@ -683,15 +683,15 @@
         <x:v>任务与规则</x:v>
       </x:c>
       <x:c r="B15" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A15)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A15)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C15" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A15)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A15)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D15" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A15)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A15)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="E15" s="3"/>
@@ -704,15 +704,15 @@
         <x:v>底库与识别</x:v>
       </x:c>
       <x:c r="B16" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A16)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A16)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C16" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A16)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A16)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="D16" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A16)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A16)</x:f>
         <x:v>26</x:v>
       </x:c>
       <x:c r="E16" s="3"/>
@@ -725,15 +725,15 @@
         <x:v>图片分析</x:v>
       </x:c>
       <x:c r="B17" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A17)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A17)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="C17" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A17)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A17)</x:f>
         <x:v>13</x:v>
       </x:c>
       <x:c r="D17" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A17)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A17)</x:f>
         <x:v>21</x:v>
       </x:c>
       <x:c r="E17" s="3"/>
@@ -746,15 +746,15 @@
         <x:v>大模型算法</x:v>
       </x:c>
       <x:c r="B18" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A18)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A18)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C18" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A18)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A18)</x:f>
         <x:v>22</x:v>
       </x:c>
       <x:c r="D18" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A18)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A18)</x:f>
         <x:v>40</x:v>
       </x:c>
       <x:c r="E18" s="3"/>
@@ -767,20 +767,20 @@
         <x:v>事件与展示</x:v>
       </x:c>
       <x:c r="B19" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A19)</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A19)</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C19" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A19)</x:f>
-        <x:v>13</x:v>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A19)</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D19" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A19)</x:f>
-        <x:v>22</x:v>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A19)</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E19" s="3"/>
       <x:c r="F19" s="3" t="str">
-        <x:v>单/四窗预览与叠加；新告警详情；首页统计核对。</x:v>
+        <x:v>单/四窗预览与叠加；新告警详情；事件上报本地/接口大模型审核；首页统计。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="38" customHeight="1">
@@ -788,20 +788,20 @@
         <x:v>数据对接</x:v>
       </x:c>
       <x:c r="B20" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A20)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A20)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C20" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A20)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A20)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D20" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A20)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A20)</x:f>
         <x:v>16</x:v>
       </x:c>
       <x:c r="E20" s="3"/>
       <x:c r="F20" s="3" t="str">
-        <x:v>HTTP/MQTT各核对1条新告警；MQTT加只读响应。</x:v>
+        <x:v>HTTP新告警；MQTT注册、心跳及只读请求应答。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
@@ -809,15 +809,15 @@
         <x:v>系统管理</x:v>
       </x:c>
       <x:c r="B21" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A21)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A21)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C21" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A21)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A21)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D21" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A21)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A21)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="E21" s="3"/>
@@ -830,15 +830,15 @@
         <x:v>必要补充</x:v>
       </x:c>
       <x:c r="B22" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A22)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A22)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C22" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A22)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A22)</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="D22" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A22)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A22)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E22" s="3"/>
@@ -851,15 +851,15 @@
         <x:v>收尾交付</x:v>
       </x:c>
       <x:c r="B23" s="3" t="n">
-        <x:f>COUNTIFS('主要用例'!B5:B32,A23)</x:f>
+        <x:f>COUNTIFS('主要用例'!B5:B33,A23)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!F5:F32,'主要用例'!B5:B32,A23)</x:f>
+        <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A23)</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="D23" s="3" t="n">
-        <x:f>SUMIFS('主要用例'!G5:G32,'主要用例'!B5:B32,A23)</x:f>
+        <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A23)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="3"/>
@@ -1266,7 +1266,7 @@
         <x:v>USB 摄像头发现、预览及运行算法</x:v>
       </x:c>
       <x:c r="D13" s="3" t="str">
-        <x:v>用户将 USB 摄像头接入被测盒子；开测前确认设备已识别、产品支持该输入，并记录设备节点或唯一标识。使用已就绪基础检测场景。</x:v>
+        <x:v>USB 摄像头为必测资源，现有硬件开测时核对设备枚举、标识和实时画面；使用已就绪基础检测场景。不得沿用历史“资源不足/暂不测试”跳过；异常需保存本轮证据。</x:v>
       </x:c>
       <x:c r="E13" s="3" t="str">
         <x:v>DUT;USB-CAMERA;MODEL-INVENTORY</x:v>
@@ -1773,10 +1773,10 @@
         <x:v>数据对接</x:v>
       </x:c>
       <x:c r="C28" s="8" t="str">
-        <x:v>MQTT 注册、业务响应和告警</x:v>
+        <x:v>MQTT 注册、心跳与业务响应</x:v>
       </x:c>
       <x:c r="D28" s="8" t="str">
-        <x:v>隔离Broker及订阅端可用；按当前协议确定topic、设备标识和心跳周期。</x:v>
+        <x:v>隔离 Broker 及订阅端可用；按当前控制协议确定 topic、设备标识和心跳周期。主动告警由 HTTP 推送，在 Q19 验证。</x:v>
       </x:c>
       <x:c r="E28" s="8" t="str">
         <x:v>DUT;MQTT-BROKER;PUSH-AUTHORIZATION</x:v>
@@ -1797,7 +1797,9 @@
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K28" s="15" t="str"/>
-      <x:c r="L28" s="15" t="str"/>
+      <x:c r="L28" s="15" t="str">
+        <x:v>v0.6：按已确认的 HTTP 告警、MQTT 控制设计修正预期；不要求 MQTT 主动发布告警。</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="44" customHeight="1">
       <x:c r="A29" s="3" t="str">
@@ -1934,6 +1936,40 @@
       </x:c>
       <x:c r="K32" s="15" t="str"/>
       <x:c r="L32" s="15" t="str"/>
+    </x:row>
+    <x:row r="33" ht="150" customHeight="1">
+      <x:c r="A33" s="8" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B33" s="8" t="str">
+        <x:v>事件与展示</x:v>
+      </x:c>
+      <x:c r="C33" s="8" t="str">
+        <x:v>事件上报大模型审核（本地模型与OpenAI接口）</x:v>
+      </x:c>
+      <x:c r="D33" s="8" t="str">
+        <x:v>使用FACE-VIDEO固定视频及人工可见的人物特征正负片段；本地VLM与OpenAI接口分别预检。审核由事件上报组件执行，普通行人检测产生候选，HTTP接收就绪。</x:v>
+      </x:c>
+      <x:c r="E33" s="8" t="str">
+        <x:v>DUT;FACE-VIDEO;MODEL-INVENTORY;VLM-MODEL;OPENAI-VLM;HTTP-RECEIVER;PUSH-AUTHORIZATION</x:v>
+      </x:c>
+      <x:c r="F33" s="14" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G33" s="14" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H33" s="8" t="str">
+        <x:v>停止并删除本轮视频任务、临时通道与复制场景；恢复原推送、审核参数和视频播放配置。保留原有业务及历史事件，不修改共享模型服务。</x:v>
+      </x:c>
+      <x:c r="I33" s="8" t="str">
+        <x:v>EVENT-012;EVENT-013;EVENT-014</x:v>
+      </x:c>
+      <x:c r="J33" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="K33" s="15"/>
+      <x:c r="L33" s="15"/>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="J5:J32">
@@ -1948,7 +1984,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re41452dbcac24286"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7eddc8026ba4afc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3926,13 +3962,13 @@
         <x:v>Q20-S03</x:v>
       </x:c>
       <x:c r="C87" s="3" t="str">
-        <x:v>触发一条新告警，从订阅端核对业务消息及媒体字段；恢复原配置。</x:v>
+        <x:v>核对只读设备信息响应中的业务结果；停止本轮订阅/请求，恢复原 MQTT 配置并刷新读回。</x:v>
       </x:c>
       <x:c r="D87" s="3" t="str">
-        <x:v>收到真实新告警且字段与事件中心一致；恢复配置可读回。</x:v>
+        <x:v>只读响应业务结果成功且内容与设备一致；原 MQTT 配置可读回。主动告警由 Q19 的 HTTP 闭环覆盖，不要求 MQTT 主动发布告警。</x:v>
       </x:c>
       <x:c r="E87" s="3" t="str">
-        <x:v>业务消息、事件ID和恢复证据。</x:v>
+        <x:v>只读业务响应、设备信息核对结果、恢复配置证据。</x:v>
       </x:c>
       <x:c r="F87" s="15" t="str"/>
       <x:c r="G87" s="15" t="str">
@@ -4216,6 +4252,167 @@
       </x:c>
       <x:c r="H99" s="15" t="str"/>
       <x:c r="I99" s="15" t="str"/>
+    </x:row>
+    <x:row r="100" ht="127.5" customHeight="1">
+      <x:c r="A100" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B100" s="3" t="str">
+        <x:v>Q29-S01</x:v>
+      </x:c>
+      <x:c r="C100" s="3" t="str">
+        <x:v>核对 FACE-VIDEO 固定视频和本地/接口两种审核资源；人工标注匹配与不匹配人物ROI、时间段。提示词可用“穿红色衣服的人”，缺红衣正例则选择实际可见特征。</x:v>
+      </x:c>
+      <x:c r="D100" s="3" t="str">
+        <x:v>正负事实可从当前目标裁剪图独立确认；未出现的特征不编造正例；两种模式分别记录资源与结果，缺一不影响另一模式可执行步骤。</x:v>
+      </x:c>
+      <x:c r="E100" s="3" t="str">
+        <x:v>视频哈希、片段/帧/目标框标注、提示词、本地模型及脱敏接口资源。</x:v>
+      </x:c>
+      <x:c r="F100" s="15"/>
+      <x:c r="G100" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H100" s="15"/>
+      <x:c r="I100" s="15"/>
+    </x:row>
+    <x:row r="101" ht="127.5" customHeight="1">
+      <x:c r="A101" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B101" s="3" t="str">
+        <x:v>Q29-S02</x:v>
+      </x:c>
+      <x:c r="C101" s="3" t="str">
+        <x:v>复制行人检测/区域入侵场景，使用事件上报组件BA_00004；关闭审核，从相同起点重播正负片段建立基线。</x:v>
+      </x:c>
+      <x:c r="D101" s="3" t="str">
+        <x:v>正负候选均实际触发基线上报；固定ROI、告警间隔、去重和播放次数。独立VLM节点输出不能代替事件上报组件审核。</x:v>
+      </x:c>
+      <x:c r="E101" s="3" t="str">
+        <x:v>场景链、组件配置、候选目标/帧、基线事件与HTTP接收记录。</x:v>
+      </x:c>
+      <x:c r="F101" s="15"/>
+      <x:c r="G101" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H101" s="15"/>
+      <x:c r="I101" s="15"/>
+    </x:row>
+    <x:row r="102" ht="127.5" customHeight="1">
+      <x:c r="A102" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B102" s="3" t="str">
+        <x:v>Q29-S03</x:v>
+      </x:c>
+      <x:c r="C102" s="3" t="str">
+        <x:v>开启本地模型审核，填写人物特征提示词并保存刷新；串行重播正负片段，逐目标对账审核日志、事件中心及HTTP接收。</x:v>
+      </x:c>
+      <x:c r="D102" s="3" t="str">
+        <x:v>本地模式真实执行：“是”对应事件放行，“否”有审核过滤证据且无该候选普通告警。不能以无检测或去重冒充审核过滤。</x:v>
+      </x:c>
+      <x:c r="E102" s="3" t="str">
+        <x:v>本地模式配置、目标裁剪图、审核结果、事件ID和HTTP对账。</x:v>
+      </x:c>
+      <x:c r="F102" s="15"/>
+      <x:c r="G102" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H102" s="15"/>
+      <x:c r="I102" s="15"/>
+    </x:row>
+    <x:row r="103" ht="127.5" customHeight="1">
+      <x:c r="A103" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B103" s="3" t="str">
+        <x:v>Q29-S04</x:v>
+      </x:c>
+      <x:c r="C103" s="3" t="str">
+        <x:v>切换OpenAI兼容接口模式，按私有配置填写基地址、served-model-name与认证；保存刷新，按服务并发限制串行重播同一正负片段。</x:v>
+      </x:c>
+      <x:c r="D103" s="3" t="str">
+        <x:v>图像请求实际发往所配服务，“是”放行、“否”过滤；结果关联当前目标与帧，接口请求失败不当作否定判断。</x:v>
+      </x:c>
+      <x:c r="E103" s="3" t="str">
+        <x:v>脱敏模式/模型配置、服务图像请求应答、审核过滤记录和事件/HTTP关联。</x:v>
+      </x:c>
+      <x:c r="F103" s="15"/>
+      <x:c r="G103" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H103" s="15"/>
+      <x:c r="I103" s="15"/>
+    </x:row>
+    <x:row r="104" ht="127.5" customHeight="1">
+      <x:c r="A104" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B104" s="3" t="str">
+        <x:v>Q29-S05</x:v>
+      </x:c>
+      <x:c r="C104" s="3" t="str">
+        <x:v>把同一目标的匹配提示词改成明显不匹配的衣着特征，保存刷新并停启任务，再重播同一片段；分别核对已测两种模式。</x:v>
+      </x:c>
+      <x:c r="D104" s="3" t="str">
+        <x:v>回读和实际审核使用新提示词；结果符合人工标注且不是上次缓存。同帧其他人的特征不替代当前目标。</x:v>
+      </x:c>
+      <x:c r="E104" s="3" t="str">
+        <x:v>修改前后提示词、停启与实际请求、目标ROI、判断及事件变化。</x:v>
+      </x:c>
+      <x:c r="F104" s="15"/>
+      <x:c r="G104" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H104" s="15"/>
+      <x:c r="I104" s="15"/>
+    </x:row>
+    <x:row r="105" ht="127.5" customHeight="1">
+      <x:c r="A105" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B105" s="3" t="str">
+        <x:v>Q29-S06</x:v>
+      </x:c>
+      <x:c r="C105" s="3" t="str">
+        <x:v>仅在本轮接口配置中暂填无效API Key，触发一次审核；记录认证失败后恢复正确值并重播正负片段。</x:v>
+      </x:c>
+      <x:c r="D105" s="3" t="str">
+        <x:v>认证错误与模型否定分开记录；当前普通接口路径错误时降级放行并留日志，恢复后真实审核再次生效，其他业务不受影响。</x:v>
+      </x:c>
+      <x:c r="E105" s="3" t="str">
+        <x:v>脱敏认证错误、故障期事件、恢复配置及恢复后正负审核证据。</x:v>
+      </x:c>
+      <x:c r="F105" s="15"/>
+      <x:c r="G105" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H105" s="15"/>
+      <x:c r="I105" s="15"/>
+    </x:row>
+    <x:row r="106" ht="127.5" customHeight="1">
+      <x:c r="A106" s="3" t="str">
+        <x:v>Q29</x:v>
+      </x:c>
+      <x:c r="B106" s="3" t="str">
+        <x:v>Q29-S07</x:v>
+      </x:c>
+      <x:c r="C106" s="3" t="str">
+        <x:v>关闭审核再重播原负例确认基线上报恢复；停止删除本轮任务、通道和复制场景，恢复原推送与参数。</x:v>
+      </x:c>
+      <x:c r="D106" s="3" t="str">
+        <x:v>关闭审核后恢复原上报规则；两种模式结果分别留证。清理不影响原业务，不修改或停止共享模型服务。</x:v>
+      </x:c>
+      <x:c r="E106" s="3" t="str">
+        <x:v>开关关闭后的事件、两种模式结论及清理恢复清单。</x:v>
+      </x:c>
+      <x:c r="F106" s="15"/>
+      <x:c r="G106" s="15" t="str">
+        <x:v>未执行</x:v>
+      </x:c>
+      <x:c r="H106" s="15"/>
+      <x:c r="I106" s="15"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -4225,7 +4422,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2b7724b3fd145c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb366a5cee4e7479d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4488,7 +4685,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a34ebdf0ecb49ff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1fa59185af24369"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4530,21 +4727,21 @@
         <x:v>评审意见</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="44" customHeight="1">
+    <x:row r="5" ht="60" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>耗时口径</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>141–232分钟为初始估算，约2小时21分至3小时52分；尚未用此版计时实跑。模型导入与首次初始化、首次配置、部署服务、完整包校验、下载、重试和排障另计。</x:v>
+        <x:v>157–260分钟为设计估算，尚未用此版计时实跑。首次模型初始化、配置、服务部署、下载、重试及排障另计。</x:v>
       </x:c>
       <x:c r="C5" s="15" t="str"/>
     </x:row>
-    <x:row r="6" ht="36" customHeight="1">
+    <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="8" t="str">
         <x:v>提速方式</x:v>
       </x:c>
       <x:c r="B6" s="8" t="str">
-        <x:v>复用短视频、场景、底库和事件；按接入方式逐路串行；控制素材和模型大小；不再展开327条全量用例及其参数/接口矩阵。</x:v>
+        <x:v>复用短视频、场景、底库和事件；接入方式与审核模式逐项串行；不展开331条全量用例及其矩阵。</x:v>
       </x:c>
       <x:c r="C6" s="15" t="str"/>
     </x:row>
@@ -4557,12 +4754,12 @@
       </x:c>
       <x:c r="C7" s="15" t="str"/>
     </x:row>
-    <x:row r="8" ht="44" customHeight="1">
+    <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="8" t="str">
         <x:v>执行顺序</x:v>
       </x:c>
       <x:c r="B8" s="8" t="str">
-        <x:v>Q01准备；Q02–Q03资源管理；Q04–Q08和Q25输入；Q09–Q10任务；Q11–Q16识别与图片；Q26–Q27大模型；Q17/Q28/Q18事件与大屏；Q19–Q20推送；Q21–Q24系统及收尾。</x:v>
+        <x:v>Q01准备；Q02–Q03资源；Q04–Q08和Q25输入；Q09–Q10任务；Q11–Q16识别与图片；Q26–Q27大模型；Q29事件上报审核；Q17/Q28/Q18事件展示；Q19–Q20推送；Q21–Q24收尾。</x:v>
       </x:c>
       <x:c r="C8" s="15" t="str"/>
     </x:row>
@@ -4593,12 +4790,12 @@
       </x:c>
       <x:c r="C11" s="15" t="str"/>
     </x:row>
-    <x:row r="12" ht="44" customHeight="1">
+    <x:row r="12" ht="60" customHeight="1">
       <x:c r="A12" s="8" t="str">
         <x:v>精度边界</x:v>
       </x:c>
       <x:c r="B12" s="8" t="str">
-        <x:v>VLM 与 DINO 用人工可见的正负固定样本判定基本功能，不宣称精度达标；USB、VLM、DINO 已纳入必测，缺可运行模型记阻塞。其他无模型场景、音柱和授权验收仍排除。</x:v>
+        <x:v>VLM、DINO及事件上报审核用人工可见正负样本验证基本功能，不宣称精度达标。USB必测；本地/接口审核独立记录，缺项只阻塞对应步骤。</x:v>
       </x:c>
       <x:c r="C12" s="15" t="str"/>
     </x:row>
@@ -4611,30 +4808,30 @@
       </x:c>
       <x:c r="C13" s="15" t="str"/>
     </x:row>
-    <x:row r="14" ht="36" customHeight="1">
+    <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="8" t="str">
         <x:v>与全量库关系</x:v>
       </x:c>
       <x:c r="B14" s="8" t="str">
-        <x:v>全量库版本1.4.0；“主要用例”按编号保留来源映射，覆盖范围经过裁剪，不能把快速通过回填为原全量用例通过。</x:v>
+        <x:v>全量库版本1.6.0；保留编号来源映射，快速通过不回填全量用例通过。</x:v>
       </x:c>
       <x:c r="C14" s="15" t="str"/>
     </x:row>
-    <x:row r="15" ht="36" customHeight="1">
+    <x:row r="15" ht="60" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>实施状态</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
-        <x:v>此文件是独立评审稿，尚未接入customer_journey.py执行队列。评审确认后实现quick模式，仍复用资源包和逐步记录机制。</x:v>
+        <x:v>正式快测用例库，已接入customer_journey.py；每轮冻结副本，执行结果另存。</x:v>
       </x:c>
       <x:c r="C15" s="15" t="str"/>
     </x:row>
-    <x:row r="16" ht="36" customHeight="1">
+    <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="8" t="str">
         <x:v>评审决策1</x:v>
       </x:c>
       <x:c r="B16" s="8" t="str">
-        <x:v>默认采用28条/约2小时21分至3小时52分是否合适？更短预算应明确减少范围，不能隐去协议或模块。</x:v>
+        <x:v>当前29条核心用例，预计157–260分钟；若减少范围须明确列出未执行项。</x:v>
       </x:c>
       <x:c r="C16" s="15" t="str"/>
     </x:row>
@@ -4674,12 +4871,12 @@
       </x:c>
       <x:c r="C20" s="15" t="str"/>
     </x:row>
-    <x:row r="21" ht="44" customHeight="1">
+    <x:row r="21" ht="60" customHeight="1">
       <x:c r="A21" s="3" t="str">
         <x:v>USB资源</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
-        <x:v>USB-CAMERA 为外接硬件，不需要复制进素材包；资源配置已取消旧排除，预检提示待核实，正式开测以盒子端枚举和画面为准。</x:v>
+        <x:v>USB-CAMERA 已纳入必测，硬件资源就绪状态维护在私有配置。每轮仍核对设备列表、实时画面、算法输出和启停恢复；旧缺口不构成本轮免测依据。</x:v>
       </x:c>
       <x:c r="C21" s="15" t="str"/>
     </x:row>
@@ -4692,12 +4889,12 @@
       </x:c>
       <x:c r="C22" s="15" t="str"/>
     </x:row>
-    <x:row r="23" ht="44" customHeight="1">
+    <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="3" t="str">
         <x:v>大模型资源</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
-        <x:v>VLM-MODEL 与 DINO-MODEL 分别预检。现有 BM1688 GroundingDINO 包是候选；Qwen 原始 bmodel/配置尚不能证明可导入。开测前记录模型包、词表/分词器、设备加载状态、正负样本哈希及提示词；缺项只阻塞 Q26/Q27 对应项。</x:v>
+        <x:v>本地VLM、DINO与OPENAI-VLM分别预检；接口审核核对实际served-model-name、认证、图像输入和并发限制。资源地址、模型与密钥放私有配置，缺项只影响对应模式。</x:v>
       </x:c>
       <x:c r="C23" s="15" t="str"/>
     </x:row>
@@ -4719,19 +4916,19 @@
       </x:c>
       <x:c r="C25" s="15" t="str"/>
     </x:row>
-    <x:row r="26" ht="44" customHeight="1">
+    <x:row r="26" ht="60" customHeight="1">
       <x:c r="A26" s="8" t="str">
         <x:v>资料来源</x:v>
       </x:c>
       <x:c r="B26" s="8" t="str">
-        <x:v>仓库test/customer-journey/CosmoEdge-客户旅程测试用例.xlsx（1.4.0）及其suite.json；用户本次范围和此前明确排除项。</x:v>
+        <x:v>正式全量用例库1.6.0、当前组件实现与用户确认的USB必测、固定视频及接口审核范围。</x:v>
       </x:c>
       <x:c r="C26" s="15" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31a6607c72a14748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca257cbc92b142c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: clean picture presets and legacy OBB template fields
Remove bundled picture scenes while retaining reusable templates. Clean legacy OBB metadata for three platforms and add customer journey coverage for OBB thresholds and parameter persistence.
</commit_message>
<xml_diff>
--- a/test/customer-journey/CosmoEdge-主要功能客户旅程测试用例.xlsx
+++ b/test/customer-journey/CosmoEdge-主要功能客户旅程测试用例.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评审总览" sheetId="1" r:id="R4e2e12dec86c44b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主要用例" sheetId="2" r:id="Reb05f24b4b734d80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤与验收" sheetId="3" r:id="R23f294e649194cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="按需补测" sheetId="4" r:id="Ra763ecfcb5974a60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="范围与评审" sheetId="5" r:id="R9023807993d24ff5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评审总览" sheetId="1" r:id="R01543374d3264a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主要用例" sheetId="2" r:id="Rd6611126b8a44e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步骤与验收" sheetId="3" r:id="Rf18455718b9642e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="按需补测" sheetId="4" r:id="Raceafb6590e74d11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="范围与评审" sheetId="5" r:id="R682e7dd91ba9449b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +472,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="16" t="str">
-        <x:v>v0.7 已确认快测用例 · 2026-10-19 · 用例定义，实测结果另存</x:v>
+        <x:v>v0.8 已确认快测用例 · 2026-10-19 · 用例定义，实测结果另存</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -533,7 +533,7 @@
       </x:c>
       <x:c r="B7" s="3" t="n">
         <x:f>SUM('主要用例'!F5:F33)</x:f>
-        <x:v>157</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3" t="str">
@@ -553,7 +553,7 @@
       </x:c>
       <x:c r="B8" s="3" t="n">
         <x:f>SUM('主要用例'!G5:G33)</x:f>
-        <x:v>260</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3" t="str">
@@ -730,11 +730,11 @@
       </x:c>
       <x:c r="C17" s="3" t="n">
         <x:f>SUMIFS('主要用例'!F5:F33,'主要用例'!B5:B33,A17)</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D17" s="3" t="n">
         <x:f>SUMIFS('主要用例'!G5:G33,'主要用例'!B5:B33,A17)</x:f>
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E17" s="3"/>
       <x:c r="F17" s="3" t="str">
@@ -1459,7 +1459,7 @@
       <x:c r="K18" s="15" t="str"/>
       <x:c r="L18" s="15" t="str"/>
     </x:row>
-    <x:row r="19" ht="44" customHeight="1">
+    <x:row r="19" ht="65" customHeight="1">
       <x:c r="A19" s="3" t="str">
         <x:v>Q14</x:v>
       </x:c>
@@ -1470,28 +1470,30 @@
         <x:v>单图、批量图片和临时参数</x:v>
       </x:c>
       <x:c r="D19" s="3" t="str">
-        <x:v>选2张可解码、目标清晰的图片；Q03 图片场景可用，或使用已存在的等价测试场景。</x:v>
+        <x:v>选2张可解码、目标清晰的图片；Q03图片场景可用。核对模型类别，准备分值介于0和1的稳定目标用于阈值对照；OBB已部署时优先抽样，专项另执行ALG-38874。</x:v>
       </x:c>
       <x:c r="E19" s="3" t="str">
-        <x:v>DUT;IMAGE-MEDIA</x:v>
+        <x:v>DUT;IMAGE-MEDIA;MODEL-INVENTORY</x:v>
       </x:c>
       <x:c r="F19" s="13" t="n">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="G19" s="13" t="n">
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
         <x:v>清空本轮图片及临时设置；任务按页面/接口生命周期释放。</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>IMAGE-001;IMAGE-002;IMAGE-003;IMAGE-011;SCENE-010</x:v>
+        <x:v>IMAGE-001;IMAGE-002;IMAGE-003;IMAGE-011;SCENE-010;IMAGE-007;ALG-38874</x:v>
       </x:c>
       <x:c r="J19" s="15" t="str">
         <x:v>未执行</x:v>
       </x:c>
       <x:c r="K19" s="15" t="str"/>
-      <x:c r="L19" s="15" t="str"/>
+      <x:c r="L19" s="15" t="str">
+        <x:v>v0.8补充旧字段与直接阈值对照；这里只抽样，不能替代ALG-38874全项验收。</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="44" customHeight="1">
       <x:c r="A20" s="8" t="str">
@@ -1984,7 +1986,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7eddc8026ba4afc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60c143b7df11423f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3195,7 +3197,7 @@
       <x:c r="H53" s="15" t="str"/>
       <x:c r="I53" s="15" t="str"/>
     </x:row>
-    <x:row r="54" ht="36" customHeight="1">
+    <x:row r="54" ht="50" customHeight="1">
       <x:c r="A54" s="8" t="str">
         <x:v>Q14</x:v>
       </x:c>
@@ -3203,13 +3205,13 @@
         <x:v>Q14-S01</x:v>
       </x:c>
       <x:c r="C54" s="8" t="str">
-        <x:v>选择图片场景，上传1张图片并提交分析。</x:v>
+        <x:v>选择图片场景，检查参数面板和编排，再上传1张图片提交分析。</x:v>
       </x:c>
       <x:c r="D54" s="8" t="str">
-        <x:v>场景可选；输出目标/业务结果与当前图片对应；结果未沿用旧图片。</x:v>
+        <x:v>无视频区域/布防配置和无效置信度偏移；直接置信度阈值可用。输出与当前图片对应；若为OBB，核对旋转框和原图，不沿用旧结果。</x:v>
       </x:c>
       <x:c r="E54" s="8" t="str">
-        <x:v>输入哈希、场景ID、结果和标注图。</x:v>
+        <x:v>参数与编排截图、输入哈希、场景及模型标识、原始结果与标注图。</x:v>
       </x:c>
       <x:c r="F54" s="15" t="str"/>
       <x:c r="G54" s="15" t="str">
@@ -3241,7 +3243,7 @@
       <x:c r="H55" s="15" t="str"/>
       <x:c r="I55" s="15" t="str"/>
     </x:row>
-    <x:row r="56" ht="44" customHeight="1">
+    <x:row r="56" ht="65" customHeight="1">
       <x:c r="A56" s="8" t="str">
         <x:v>Q14</x:v>
       </x:c>
@@ -3249,13 +3251,13 @@
         <x:v>Q14-S03</x:v>
       </x:c>
       <x:c r="C56" s="8" t="str">
-        <x:v>修改1个临时分析参数并提交；刷新或新开同场景，检查默认值。</x:v>
+        <x:v>记录稳定目标分值，用其两侧的直接置信度阈值重测同一图；刷新检查默认值。保存并重新打开场景，再检查参数声明。</x:v>
       </x:c>
       <x:c r="D56" s="8" t="str">
-        <x:v>临时值参与本次分析；场景/任务默认值未被永久改写；再次分析可用。</x:v>
+        <x:v>低阈值保留、高阈值过滤同一目标；临时值不改默认，保存重开不恢复旧字段。缺边界样本明确记录缺口；不能只以请求成功判定阈值生效。</x:v>
       </x:c>
       <x:c r="E56" s="8" t="str">
-        <x:v>临时请求、默认值和再次分析结果。</x:v>
+        <x:v>同一目标两次阈值、请求与返回对照；默认值回读；保存重开后的参数截图。</x:v>
       </x:c>
       <x:c r="F56" s="15" t="str"/>
       <x:c r="G56" s="15" t="str">
@@ -4422,7 +4424,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb366a5cee4e7479d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd415d8ce9c89455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4685,7 +4687,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1fa59185af24369"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e23897c5a7e4053"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4928,7 +4930,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca257cbc92b142c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95389c2c329e48b4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>